<commit_message>
Add Agent 5 QA adjudicator, and redesign the dashboard
</commit_message>
<xml_diff>
--- a/out/S01_campus_cafeteria_experience/agent3/agent3_review.xlsx
+++ b/out/S01_campus_cafeteria_experience/agent3/agent3_review.xlsx
@@ -16317,7 +16317,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>EX-e444d15cd5</t>
+          <t>EX-83fb5e05d4</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -16367,7 +16367,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>EX-e444d15cd5</t>
+          <t>EX-83fb5e05d4</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -16417,7 +16417,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>EX-e444d15cd5</t>
+          <t>EX-83fb5e05d4</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -16451,7 +16451,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>EX-e444d15cd5</t>
+          <t>EX-83fb5e05d4</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -16501,7 +16501,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>EX-e444d15cd5</t>
+          <t>EX-83fb5e05d4</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -16551,7 +16551,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>EX-e444d15cd5</t>
+          <t>EX-83fb5e05d4</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -16601,7 +16601,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>EX-e444d15cd5</t>
+          <t>EX-83fb5e05d4</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -16651,7 +16651,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>EX-e444d15cd5</t>
+          <t>EX-83fb5e05d4</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -16701,7 +16701,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>EX-e444d15cd5</t>
+          <t>EX-83fb5e05d4</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -16751,7 +16751,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>EX-e444d15cd5</t>
+          <t>EX-83fb5e05d4</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -16801,7 +16801,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>EX-e444d15cd5</t>
+          <t>EX-83fb5e05d4</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -16851,7 +16851,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>EX-e444d15cd5</t>
+          <t>EX-83fb5e05d4</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -16885,7 +16885,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>EX-13ff676266</t>
+          <t>EX-4ec3f9bc99</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -16935,7 +16935,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>EX-13ff676266</t>
+          <t>EX-4ec3f9bc99</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -16985,7 +16985,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>EX-13ff676266</t>
+          <t>EX-4ec3f9bc99</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -17019,7 +17019,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>EX-13ff676266</t>
+          <t>EX-4ec3f9bc99</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -17069,7 +17069,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>EX-13ff676266</t>
+          <t>EX-4ec3f9bc99</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -17119,7 +17119,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>EX-13ff676266</t>
+          <t>EX-4ec3f9bc99</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -17169,7 +17169,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>EX-13ff676266</t>
+          <t>EX-4ec3f9bc99</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -17219,7 +17219,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>EX-13ff676266</t>
+          <t>EX-4ec3f9bc99</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -17269,7 +17269,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>EX-13ff676266</t>
+          <t>EX-4ec3f9bc99</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -17319,7 +17319,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>EX-13ff676266</t>
+          <t>EX-4ec3f9bc99</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -17369,7 +17369,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>EX-13ff676266</t>
+          <t>EX-4ec3f9bc99</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -17419,7 +17419,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>EX-13ff676266</t>
+          <t>EX-4ec3f9bc99</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -17453,7 +17453,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>EX-36fbba288b</t>
+          <t>EX-5e147c7716</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -17503,7 +17503,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>EX-36fbba288b</t>
+          <t>EX-5e147c7716</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -17553,7 +17553,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>EX-36fbba288b</t>
+          <t>EX-5e147c7716</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -17587,7 +17587,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>EX-36fbba288b</t>
+          <t>EX-5e147c7716</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -17637,7 +17637,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>EX-36fbba288b</t>
+          <t>EX-5e147c7716</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -17687,7 +17687,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>EX-36fbba288b</t>
+          <t>EX-5e147c7716</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -17737,7 +17737,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>EX-36fbba288b</t>
+          <t>EX-5e147c7716</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -17787,7 +17787,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>EX-36fbba288b</t>
+          <t>EX-5e147c7716</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -17837,7 +17837,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>EX-36fbba288b</t>
+          <t>EX-5e147c7716</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -17887,7 +17887,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>EX-36fbba288b</t>
+          <t>EX-5e147c7716</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -17937,7 +17937,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>EX-36fbba288b</t>
+          <t>EX-5e147c7716</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -17987,7 +17987,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>EX-36fbba288b</t>
+          <t>EX-5e147c7716</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -18021,7 +18021,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>EX-f7fceef0cf</t>
+          <t>EX-afe8f4bfe5</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -18071,7 +18071,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>EX-f7fceef0cf</t>
+          <t>EX-afe8f4bfe5</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -18121,7 +18121,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>EX-f7fceef0cf</t>
+          <t>EX-afe8f4bfe5</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -18155,7 +18155,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>EX-f7fceef0cf</t>
+          <t>EX-afe8f4bfe5</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -18205,7 +18205,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>EX-f7fceef0cf</t>
+          <t>EX-afe8f4bfe5</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -18255,7 +18255,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>EX-f7fceef0cf</t>
+          <t>EX-afe8f4bfe5</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -18305,7 +18305,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>EX-f7fceef0cf</t>
+          <t>EX-afe8f4bfe5</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -18355,7 +18355,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>EX-f7fceef0cf</t>
+          <t>EX-afe8f4bfe5</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -18405,7 +18405,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>EX-f7fceef0cf</t>
+          <t>EX-afe8f4bfe5</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -18455,7 +18455,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>EX-f7fceef0cf</t>
+          <t>EX-afe8f4bfe5</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -18505,7 +18505,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>EX-f7fceef0cf</t>
+          <t>EX-afe8f4bfe5</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -18555,7 +18555,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>EX-f7fceef0cf</t>
+          <t>EX-afe8f4bfe5</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -18589,7 +18589,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>EX-a214f02dcd</t>
+          <t>EX-3eb0769072</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -18639,7 +18639,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>EX-a214f02dcd</t>
+          <t>EX-3eb0769072</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -18689,7 +18689,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>EX-a214f02dcd</t>
+          <t>EX-3eb0769072</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -18723,7 +18723,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>EX-a214f02dcd</t>
+          <t>EX-3eb0769072</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -18773,7 +18773,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>EX-a214f02dcd</t>
+          <t>EX-3eb0769072</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -18823,7 +18823,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>EX-a214f02dcd</t>
+          <t>EX-3eb0769072</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -18873,7 +18873,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>EX-a214f02dcd</t>
+          <t>EX-3eb0769072</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -18923,7 +18923,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>EX-a214f02dcd</t>
+          <t>EX-3eb0769072</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -18973,7 +18973,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>EX-a214f02dcd</t>
+          <t>EX-3eb0769072</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -19023,7 +19023,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>EX-a214f02dcd</t>
+          <t>EX-3eb0769072</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -19073,7 +19073,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>EX-a214f02dcd</t>
+          <t>EX-3eb0769072</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -19123,7 +19123,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>EX-a214f02dcd</t>
+          <t>EX-3eb0769072</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -19157,7 +19157,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>EX-f02a205850</t>
+          <t>EX-1e2be181e7</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -19207,7 +19207,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>EX-f02a205850</t>
+          <t>EX-1e2be181e7</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -19257,7 +19257,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>EX-f02a205850</t>
+          <t>EX-1e2be181e7</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -19291,7 +19291,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>EX-f02a205850</t>
+          <t>EX-1e2be181e7</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -19341,7 +19341,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>EX-f02a205850</t>
+          <t>EX-1e2be181e7</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -19391,7 +19391,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>EX-f02a205850</t>
+          <t>EX-1e2be181e7</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -19441,7 +19441,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>EX-f02a205850</t>
+          <t>EX-1e2be181e7</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -19491,7 +19491,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>EX-f02a205850</t>
+          <t>EX-1e2be181e7</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -19541,7 +19541,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>EX-f02a205850</t>
+          <t>EX-1e2be181e7</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -19591,7 +19591,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>EX-f02a205850</t>
+          <t>EX-1e2be181e7</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -19641,7 +19641,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>EX-f02a205850</t>
+          <t>EX-1e2be181e7</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -19691,7 +19691,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>EX-f02a205850</t>
+          <t>EX-1e2be181e7</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -19725,7 +19725,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>EX-17f2db79d6</t>
+          <t>EX-b24b14d127</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -19775,7 +19775,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>EX-17f2db79d6</t>
+          <t>EX-b24b14d127</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -19825,7 +19825,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>EX-17f2db79d6</t>
+          <t>EX-b24b14d127</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -19859,7 +19859,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>EX-17f2db79d6</t>
+          <t>EX-b24b14d127</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -19909,7 +19909,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>EX-17f2db79d6</t>
+          <t>EX-b24b14d127</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -19959,7 +19959,7 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>EX-17f2db79d6</t>
+          <t>EX-b24b14d127</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -20009,7 +20009,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>EX-17f2db79d6</t>
+          <t>EX-b24b14d127</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -20059,7 +20059,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>EX-17f2db79d6</t>
+          <t>EX-b24b14d127</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -20109,7 +20109,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>EX-17f2db79d6</t>
+          <t>EX-b24b14d127</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -20159,7 +20159,7 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>EX-17f2db79d6</t>
+          <t>EX-b24b14d127</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -20209,7 +20209,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>EX-17f2db79d6</t>
+          <t>EX-b24b14d127</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -20243,7 +20243,7 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>EX-0406c0b88e</t>
+          <t>EX-a99c212c1b</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -20293,7 +20293,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>EX-0406c0b88e</t>
+          <t>EX-a99c212c1b</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -20343,7 +20343,7 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>EX-0406c0b88e</t>
+          <t>EX-a99c212c1b</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -20377,7 +20377,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>EX-0406c0b88e</t>
+          <t>EX-a99c212c1b</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -20427,7 +20427,7 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>EX-0406c0b88e</t>
+          <t>EX-a99c212c1b</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -20477,7 +20477,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>EX-0406c0b88e</t>
+          <t>EX-a99c212c1b</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -20527,7 +20527,7 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>EX-0406c0b88e</t>
+          <t>EX-a99c212c1b</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -20577,7 +20577,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>EX-0406c0b88e</t>
+          <t>EX-a99c212c1b</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -20627,7 +20627,7 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>EX-0406c0b88e</t>
+          <t>EX-a99c212c1b</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -20677,7 +20677,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>EX-0406c0b88e</t>
+          <t>EX-a99c212c1b</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -20727,7 +20727,7 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>EX-0406c0b88e</t>
+          <t>EX-a99c212c1b</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -20777,7 +20777,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>EX-0406c0b88e</t>
+          <t>EX-a99c212c1b</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -20811,7 +20811,7 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>EX-2f1c4f80c4</t>
+          <t>EX-eefe0eb2e2</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -20861,7 +20861,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>EX-2f1c4f80c4</t>
+          <t>EX-eefe0eb2e2</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -20911,7 +20911,7 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>EX-2f1c4f80c4</t>
+          <t>EX-eefe0eb2e2</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -20945,7 +20945,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>EX-2f1c4f80c4</t>
+          <t>EX-eefe0eb2e2</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -20995,7 +20995,7 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>EX-2f1c4f80c4</t>
+          <t>EX-eefe0eb2e2</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -21045,7 +21045,7 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>EX-2f1c4f80c4</t>
+          <t>EX-eefe0eb2e2</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -21095,7 +21095,7 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>EX-2f1c4f80c4</t>
+          <t>EX-eefe0eb2e2</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
@@ -21145,7 +21145,7 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>EX-2f1c4f80c4</t>
+          <t>EX-eefe0eb2e2</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -21195,7 +21195,7 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>EX-2f1c4f80c4</t>
+          <t>EX-eefe0eb2e2</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
@@ -21245,7 +21245,7 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>EX-2f1c4f80c4</t>
+          <t>EX-eefe0eb2e2</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -21295,7 +21295,7 @@
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>EX-2f1c4f80c4</t>
+          <t>EX-eefe0eb2e2</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
@@ -21345,7 +21345,7 @@
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>EX-2f1c4f80c4</t>
+          <t>EX-eefe0eb2e2</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -21379,7 +21379,7 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>EX-49c22f3c37</t>
+          <t>EX-e7c2568040</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
@@ -21429,7 +21429,7 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>EX-49c22f3c37</t>
+          <t>EX-e7c2568040</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -21479,7 +21479,7 @@
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>EX-49c22f3c37</t>
+          <t>EX-e7c2568040</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
@@ -21513,7 +21513,7 @@
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>EX-49c22f3c37</t>
+          <t>EX-e7c2568040</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -21563,7 +21563,7 @@
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>EX-49c22f3c37</t>
+          <t>EX-e7c2568040</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
@@ -21613,7 +21613,7 @@
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>EX-49c22f3c37</t>
+          <t>EX-e7c2568040</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
@@ -21663,7 +21663,7 @@
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>EX-49c22f3c37</t>
+          <t>EX-e7c2568040</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
@@ -21713,7 +21713,7 @@
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>EX-49c22f3c37</t>
+          <t>EX-e7c2568040</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -21763,7 +21763,7 @@
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>EX-49c22f3c37</t>
+          <t>EX-e7c2568040</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
@@ -21813,7 +21813,7 @@
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>EX-49c22f3c37</t>
+          <t>EX-e7c2568040</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
@@ -21863,7 +21863,7 @@
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>EX-49c22f3c37</t>
+          <t>EX-e7c2568040</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
@@ -21913,7 +21913,7 @@
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>EX-49c22f3c37</t>
+          <t>EX-e7c2568040</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
@@ -21947,7 +21947,7 @@
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>EX-cf838aa662</t>
+          <t>EX-40bf3439d5</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
@@ -21997,7 +21997,7 @@
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>EX-cf838aa662</t>
+          <t>EX-40bf3439d5</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
@@ -22047,7 +22047,7 @@
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>EX-cf838aa662</t>
+          <t>EX-40bf3439d5</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
@@ -22081,7 +22081,7 @@
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>EX-cf838aa662</t>
+          <t>EX-40bf3439d5</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
@@ -22131,7 +22131,7 @@
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>EX-cf838aa662</t>
+          <t>EX-40bf3439d5</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
@@ -22181,7 +22181,7 @@
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>EX-cf838aa662</t>
+          <t>EX-40bf3439d5</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
@@ -22231,7 +22231,7 @@
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>EX-cf838aa662</t>
+          <t>EX-40bf3439d5</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
@@ -22281,7 +22281,7 @@
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>EX-cf838aa662</t>
+          <t>EX-40bf3439d5</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
@@ -22331,7 +22331,7 @@
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>EX-cf838aa662</t>
+          <t>EX-40bf3439d5</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
@@ -22381,7 +22381,7 @@
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>EX-cf838aa662</t>
+          <t>EX-40bf3439d5</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
@@ -22431,7 +22431,7 @@
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>EX-cf838aa662</t>
+          <t>EX-40bf3439d5</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
@@ -22465,7 +22465,7 @@
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>EX-10faac68cf</t>
+          <t>EX-704bb186c9</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -22515,7 +22515,7 @@
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>EX-10faac68cf</t>
+          <t>EX-704bb186c9</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
@@ -22565,7 +22565,7 @@
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>EX-10faac68cf</t>
+          <t>EX-704bb186c9</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
@@ -22599,7 +22599,7 @@
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>EX-10faac68cf</t>
+          <t>EX-704bb186c9</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
@@ -22649,7 +22649,7 @@
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>EX-10faac68cf</t>
+          <t>EX-704bb186c9</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
@@ -22699,7 +22699,7 @@
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>EX-10faac68cf</t>
+          <t>EX-704bb186c9</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
@@ -22749,7 +22749,7 @@
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>EX-10faac68cf</t>
+          <t>EX-704bb186c9</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
@@ -22799,7 +22799,7 @@
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>EX-10faac68cf</t>
+          <t>EX-704bb186c9</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
@@ -22849,7 +22849,7 @@
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>EX-10faac68cf</t>
+          <t>EX-704bb186c9</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
@@ -22899,7 +22899,7 @@
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>EX-10faac68cf</t>
+          <t>EX-704bb186c9</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
@@ -22949,7 +22949,7 @@
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>EX-10faac68cf</t>
+          <t>EX-704bb186c9</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
@@ -22983,7 +22983,7 @@
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>EX-515f124356</t>
+          <t>EX-a344c1af85</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
@@ -23033,7 +23033,7 @@
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>EX-515f124356</t>
+          <t>EX-a344c1af85</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
@@ -23083,7 +23083,7 @@
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>EX-515f124356</t>
+          <t>EX-a344c1af85</t>
         </is>
       </c>
       <c r="B145" s="2" t="inlineStr">
@@ -23117,7 +23117,7 @@
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>EX-515f124356</t>
+          <t>EX-a344c1af85</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
@@ -23167,7 +23167,7 @@
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>EX-515f124356</t>
+          <t>EX-a344c1af85</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
@@ -23217,7 +23217,7 @@
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>EX-515f124356</t>
+          <t>EX-a344c1af85</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
@@ -23267,7 +23267,7 @@
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>EX-515f124356</t>
+          <t>EX-a344c1af85</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
@@ -23317,7 +23317,7 @@
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>EX-515f124356</t>
+          <t>EX-a344c1af85</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -23367,7 +23367,7 @@
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>EX-515f124356</t>
+          <t>EX-a344c1af85</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
@@ -23417,7 +23417,7 @@
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>EX-515f124356</t>
+          <t>EX-a344c1af85</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
@@ -23467,7 +23467,7 @@
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>EX-515f124356</t>
+          <t>EX-a344c1af85</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
@@ -23517,7 +23517,7 @@
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>EX-515f124356</t>
+          <t>EX-a344c1af85</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
@@ -23551,7 +23551,7 @@
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>EX-16ed1bf3d2</t>
+          <t>EX-5ec49d8ac5</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
@@ -23601,7 +23601,7 @@
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>EX-16ed1bf3d2</t>
+          <t>EX-5ec49d8ac5</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
@@ -23651,7 +23651,7 @@
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>EX-16ed1bf3d2</t>
+          <t>EX-5ec49d8ac5</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
@@ -23685,7 +23685,7 @@
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>EX-16ed1bf3d2</t>
+          <t>EX-5ec49d8ac5</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
@@ -23735,7 +23735,7 @@
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>EX-16ed1bf3d2</t>
+          <t>EX-5ec49d8ac5</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
@@ -23785,7 +23785,7 @@
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>EX-16ed1bf3d2</t>
+          <t>EX-5ec49d8ac5</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
@@ -23835,7 +23835,7 @@
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>EX-16ed1bf3d2</t>
+          <t>EX-5ec49d8ac5</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
@@ -23885,7 +23885,7 @@
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>EX-16ed1bf3d2</t>
+          <t>EX-5ec49d8ac5</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
@@ -23935,7 +23935,7 @@
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>EX-16ed1bf3d2</t>
+          <t>EX-5ec49d8ac5</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
@@ -23985,7 +23985,7 @@
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>EX-16ed1bf3d2</t>
+          <t>EX-5ec49d8ac5</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
@@ -24035,7 +24035,7 @@
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>EX-16ed1bf3d2</t>
+          <t>EX-5ec49d8ac5</t>
         </is>
       </c>
       <c r="B165" s="2" t="inlineStr">
@@ -24085,7 +24085,7 @@
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>EX-16ed1bf3d2</t>
+          <t>EX-5ec49d8ac5</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
@@ -24119,7 +24119,7 @@
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>EX-80d557c8c4</t>
+          <t>EX-74de97f8b8</t>
         </is>
       </c>
       <c r="B167" s="2" t="inlineStr">
@@ -24169,7 +24169,7 @@
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>EX-80d557c8c4</t>
+          <t>EX-74de97f8b8</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
@@ -24219,7 +24219,7 @@
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>EX-80d557c8c4</t>
+          <t>EX-74de97f8b8</t>
         </is>
       </c>
       <c r="B169" s="2" t="inlineStr">
@@ -24253,7 +24253,7 @@
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>EX-80d557c8c4</t>
+          <t>EX-74de97f8b8</t>
         </is>
       </c>
       <c r="B170" s="2" t="inlineStr">
@@ -24303,7 +24303,7 @@
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>EX-80d557c8c4</t>
+          <t>EX-74de97f8b8</t>
         </is>
       </c>
       <c r="B171" s="2" t="inlineStr">
@@ -24353,7 +24353,7 @@
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>EX-80d557c8c4</t>
+          <t>EX-74de97f8b8</t>
         </is>
       </c>
       <c r="B172" s="2" t="inlineStr">
@@ -24403,7 +24403,7 @@
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>EX-80d557c8c4</t>
+          <t>EX-74de97f8b8</t>
         </is>
       </c>
       <c r="B173" s="2" t="inlineStr">
@@ -24453,7 +24453,7 @@
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>EX-80d557c8c4</t>
+          <t>EX-74de97f8b8</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
@@ -24503,7 +24503,7 @@
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>EX-80d557c8c4</t>
+          <t>EX-74de97f8b8</t>
         </is>
       </c>
       <c r="B175" s="2" t="inlineStr">
@@ -24553,7 +24553,7 @@
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>EX-80d557c8c4</t>
+          <t>EX-74de97f8b8</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
@@ -24603,7 +24603,7 @@
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>EX-80d557c8c4</t>
+          <t>EX-74de97f8b8</t>
         </is>
       </c>
       <c r="B177" s="2" t="inlineStr">
@@ -24653,7 +24653,7 @@
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>EX-80d557c8c4</t>
+          <t>EX-74de97f8b8</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
@@ -24687,7 +24687,7 @@
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>EX-1e9bf99444</t>
+          <t>EX-a46433941c</t>
         </is>
       </c>
       <c r="B179" s="2" t="inlineStr">
@@ -24737,7 +24737,7 @@
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>EX-1e9bf99444</t>
+          <t>EX-a46433941c</t>
         </is>
       </c>
       <c r="B180" s="2" t="inlineStr">
@@ -24787,7 +24787,7 @@
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>EX-1e9bf99444</t>
+          <t>EX-a46433941c</t>
         </is>
       </c>
       <c r="B181" s="2" t="inlineStr">
@@ -24821,7 +24821,7 @@
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>EX-f7e5521a6e</t>
+          <t>EX-1aff0c29e9</t>
         </is>
       </c>
       <c r="B182" s="2" t="inlineStr">
@@ -24871,7 +24871,7 @@
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>EX-f7e5521a6e</t>
+          <t>EX-1aff0c29e9</t>
         </is>
       </c>
       <c r="B183" s="2" t="inlineStr">
@@ -24921,7 +24921,7 @@
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>EX-f7e5521a6e</t>
+          <t>EX-1aff0c29e9</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
@@ -24955,7 +24955,7 @@
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>EX-e3802dba8c</t>
+          <t>EX-4f28a08a75</t>
         </is>
       </c>
       <c r="B185" s="2" t="inlineStr">
@@ -25005,7 +25005,7 @@
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>EX-e3802dba8c</t>
+          <t>EX-4f28a08a75</t>
         </is>
       </c>
       <c r="B186" s="2" t="inlineStr">
@@ -25055,7 +25055,7 @@
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>EX-e3802dba8c</t>
+          <t>EX-4f28a08a75</t>
         </is>
       </c>
       <c r="B187" s="2" t="inlineStr">
@@ -25089,7 +25089,7 @@
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>EX-e3802dba8c</t>
+          <t>EX-4f28a08a75</t>
         </is>
       </c>
       <c r="B188" s="2" t="inlineStr">
@@ -25139,7 +25139,7 @@
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>EX-e3802dba8c</t>
+          <t>EX-4f28a08a75</t>
         </is>
       </c>
       <c r="B189" s="2" t="inlineStr">
@@ -25189,7 +25189,7 @@
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>EX-e3802dba8c</t>
+          <t>EX-4f28a08a75</t>
         </is>
       </c>
       <c r="B190" s="2" t="inlineStr">
@@ -25239,7 +25239,7 @@
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>EX-e3802dba8c</t>
+          <t>EX-4f28a08a75</t>
         </is>
       </c>
       <c r="B191" s="2" t="inlineStr">
@@ -25289,7 +25289,7 @@
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>EX-e3802dba8c</t>
+          <t>EX-4f28a08a75</t>
         </is>
       </c>
       <c r="B192" s="2" t="inlineStr">
@@ -25339,7 +25339,7 @@
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>EX-e3802dba8c</t>
+          <t>EX-4f28a08a75</t>
         </is>
       </c>
       <c r="B193" s="2" t="inlineStr">
@@ -25389,7 +25389,7 @@
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>EX-e3802dba8c</t>
+          <t>EX-4f28a08a75</t>
         </is>
       </c>
       <c r="B194" s="2" t="inlineStr">
@@ -25439,7 +25439,7 @@
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>EX-e3802dba8c</t>
+          <t>EX-4f28a08a75</t>
         </is>
       </c>
       <c r="B195" s="2" t="inlineStr">
@@ -25489,7 +25489,7 @@
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>EX-e3802dba8c</t>
+          <t>EX-4f28a08a75</t>
         </is>
       </c>
       <c r="B196" s="2" t="inlineStr">
@@ -25523,7 +25523,7 @@
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>EX-8c6e88a595</t>
+          <t>EX-bbd4033aef</t>
         </is>
       </c>
       <c r="B197" s="2" t="inlineStr">
@@ -25573,7 +25573,7 @@
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>EX-8c6e88a595</t>
+          <t>EX-bbd4033aef</t>
         </is>
       </c>
       <c r="B198" s="2" t="inlineStr">
@@ -25623,7 +25623,7 @@
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>EX-8c6e88a595</t>
+          <t>EX-bbd4033aef</t>
         </is>
       </c>
       <c r="B199" s="2" t="inlineStr">
@@ -25657,7 +25657,7 @@
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>EX-8c6e88a595</t>
+          <t>EX-bbd4033aef</t>
         </is>
       </c>
       <c r="B200" s="2" t="inlineStr">
@@ -25707,7 +25707,7 @@
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>EX-8c6e88a595</t>
+          <t>EX-bbd4033aef</t>
         </is>
       </c>
       <c r="B201" s="2" t="inlineStr">
@@ -25757,7 +25757,7 @@
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>EX-8c6e88a595</t>
+          <t>EX-bbd4033aef</t>
         </is>
       </c>
       <c r="B202" s="2" t="inlineStr">
@@ -25807,7 +25807,7 @@
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>EX-8c6e88a595</t>
+          <t>EX-bbd4033aef</t>
         </is>
       </c>
       <c r="B203" s="2" t="inlineStr">
@@ -25849,7 +25849,7 @@
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>EX-8c6e88a595</t>
+          <t>EX-bbd4033aef</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
@@ -25899,7 +25899,7 @@
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>EX-8c6e88a595</t>
+          <t>EX-bbd4033aef</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
@@ -25949,7 +25949,7 @@
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>EX-8c6e88a595</t>
+          <t>EX-bbd4033aef</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
@@ -25999,7 +25999,7 @@
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>EX-8c6e88a595</t>
+          <t>EX-bbd4033aef</t>
         </is>
       </c>
       <c r="B207" s="2" t="inlineStr">
@@ -26049,7 +26049,7 @@
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>EX-8c6e88a595</t>
+          <t>EX-bbd4033aef</t>
         </is>
       </c>
       <c r="B208" s="2" t="inlineStr">
@@ -26083,7 +26083,7 @@
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>EX-3fda782b0c</t>
+          <t>EX-3b908df042</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
@@ -26133,7 +26133,7 @@
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>EX-3fda782b0c</t>
+          <t>EX-3b908df042</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
@@ -26183,7 +26183,7 @@
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>EX-3fda782b0c</t>
+          <t>EX-3b908df042</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
@@ -26217,7 +26217,7 @@
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>EX-3fda782b0c</t>
+          <t>EX-3b908df042</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
@@ -26267,7 +26267,7 @@
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>EX-3fda782b0c</t>
+          <t>EX-3b908df042</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
@@ -26317,7 +26317,7 @@
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>EX-3fda782b0c</t>
+          <t>EX-3b908df042</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
@@ -26367,7 +26367,7 @@
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>EX-3fda782b0c</t>
+          <t>EX-3b908df042</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
@@ -26417,7 +26417,7 @@
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>EX-3fda782b0c</t>
+          <t>EX-3b908df042</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
@@ -26467,7 +26467,7 @@
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>EX-3fda782b0c</t>
+          <t>EX-3b908df042</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
@@ -26517,7 +26517,7 @@
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>EX-3fda782b0c</t>
+          <t>EX-3b908df042</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
@@ -26567,7 +26567,7 @@
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>EX-3fda782b0c</t>
+          <t>EX-3b908df042</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
@@ -26617,7 +26617,7 @@
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>EX-3fda782b0c</t>
+          <t>EX-3b908df042</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
@@ -26651,7 +26651,7 @@
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>EX-3dc3570d3d</t>
+          <t>EX-4a2a056634</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
@@ -26701,7 +26701,7 @@
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>EX-3dc3570d3d</t>
+          <t>EX-4a2a056634</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
@@ -26751,7 +26751,7 @@
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>EX-3dc3570d3d</t>
+          <t>EX-4a2a056634</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
@@ -26785,7 +26785,7 @@
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>EX-3dc3570d3d</t>
+          <t>EX-4a2a056634</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
@@ -26835,7 +26835,7 @@
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>EX-3dc3570d3d</t>
+          <t>EX-4a2a056634</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
@@ -26885,7 +26885,7 @@
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>EX-3dc3570d3d</t>
+          <t>EX-4a2a056634</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
@@ -26935,7 +26935,7 @@
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>EX-3dc3570d3d</t>
+          <t>EX-4a2a056634</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
@@ -26985,7 +26985,7 @@
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>EX-3dc3570d3d</t>
+          <t>EX-4a2a056634</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
@@ -27035,7 +27035,7 @@
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>EX-3dc3570d3d</t>
+          <t>EX-4a2a056634</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
@@ -27085,7 +27085,7 @@
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>EX-3dc3570d3d</t>
+          <t>EX-4a2a056634</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
@@ -27135,7 +27135,7 @@
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>EX-3dc3570d3d</t>
+          <t>EX-4a2a056634</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
@@ -27185,7 +27185,7 @@
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>EX-3dc3570d3d</t>
+          <t>EX-4a2a056634</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
@@ -27219,7 +27219,7 @@
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>EX-c43adf7c1c</t>
+          <t>EX-77d29d794c</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
@@ -27269,7 +27269,7 @@
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>EX-c43adf7c1c</t>
+          <t>EX-77d29d794c</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
@@ -27319,7 +27319,7 @@
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>EX-c43adf7c1c</t>
+          <t>EX-77d29d794c</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
@@ -27353,7 +27353,7 @@
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>EX-c43adf7c1c</t>
+          <t>EX-77d29d794c</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
@@ -27403,7 +27403,7 @@
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>EX-c43adf7c1c</t>
+          <t>EX-77d29d794c</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
@@ -27453,7 +27453,7 @@
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>EX-c43adf7c1c</t>
+          <t>EX-77d29d794c</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
@@ -27503,7 +27503,7 @@
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>EX-c43adf7c1c</t>
+          <t>EX-77d29d794c</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
@@ -27553,7 +27553,7 @@
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>EX-c43adf7c1c</t>
+          <t>EX-77d29d794c</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
@@ -27603,7 +27603,7 @@
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>EX-c43adf7c1c</t>
+          <t>EX-77d29d794c</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
@@ -27653,7 +27653,7 @@
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>EX-c43adf7c1c</t>
+          <t>EX-77d29d794c</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
@@ -27703,7 +27703,7 @@
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>EX-c43adf7c1c</t>
+          <t>EX-77d29d794c</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
@@ -27753,7 +27753,7 @@
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>EX-c43adf7c1c</t>
+          <t>EX-77d29d794c</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
@@ -27787,7 +27787,7 @@
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>EX-30168f639d</t>
+          <t>EX-186eacfa0d</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
@@ -27837,7 +27837,7 @@
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>EX-30168f639d</t>
+          <t>EX-186eacfa0d</t>
         </is>
       </c>
       <c r="B246" s="2" t="inlineStr">
@@ -27887,7 +27887,7 @@
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>EX-30168f639d</t>
+          <t>EX-186eacfa0d</t>
         </is>
       </c>
       <c r="B247" s="2" t="inlineStr">
@@ -27921,7 +27921,7 @@
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>EX-30168f639d</t>
+          <t>EX-186eacfa0d</t>
         </is>
       </c>
       <c r="B248" s="2" t="inlineStr">
@@ -27971,7 +27971,7 @@
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>EX-30168f639d</t>
+          <t>EX-186eacfa0d</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
@@ -28021,7 +28021,7 @@
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>EX-30168f639d</t>
+          <t>EX-186eacfa0d</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
@@ -28071,7 +28071,7 @@
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>EX-30168f639d</t>
+          <t>EX-186eacfa0d</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
@@ -28121,7 +28121,7 @@
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>EX-30168f639d</t>
+          <t>EX-186eacfa0d</t>
         </is>
       </c>
       <c r="B252" s="2" t="inlineStr">
@@ -28171,7 +28171,7 @@
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>EX-30168f639d</t>
+          <t>EX-186eacfa0d</t>
         </is>
       </c>
       <c r="B253" s="2" t="inlineStr">
@@ -28221,7 +28221,7 @@
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>EX-30168f639d</t>
+          <t>EX-186eacfa0d</t>
         </is>
       </c>
       <c r="B254" s="2" t="inlineStr">
@@ -28271,7 +28271,7 @@
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>EX-30168f639d</t>
+          <t>EX-186eacfa0d</t>
         </is>
       </c>
       <c r="B255" s="2" t="inlineStr">
@@ -28321,7 +28321,7 @@
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>EX-30168f639d</t>
+          <t>EX-186eacfa0d</t>
         </is>
       </c>
       <c r="B256" s="2" t="inlineStr">
@@ -28355,7 +28355,7 @@
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>EX-86dd65f493</t>
+          <t>EX-9bb5386d79</t>
         </is>
       </c>
       <c r="B257" s="2" t="inlineStr">
@@ -28405,7 +28405,7 @@
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>EX-86dd65f493</t>
+          <t>EX-9bb5386d79</t>
         </is>
       </c>
       <c r="B258" s="2" t="inlineStr">
@@ -28455,7 +28455,7 @@
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>EX-86dd65f493</t>
+          <t>EX-9bb5386d79</t>
         </is>
       </c>
       <c r="B259" s="2" t="inlineStr">
@@ -28489,7 +28489,7 @@
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>EX-86dd65f493</t>
+          <t>EX-9bb5386d79</t>
         </is>
       </c>
       <c r="B260" s="2" t="inlineStr">
@@ -28539,7 +28539,7 @@
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>EX-86dd65f493</t>
+          <t>EX-9bb5386d79</t>
         </is>
       </c>
       <c r="B261" s="2" t="inlineStr">
@@ -28589,7 +28589,7 @@
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>EX-86dd65f493</t>
+          <t>EX-9bb5386d79</t>
         </is>
       </c>
       <c r="B262" s="2" t="inlineStr">
@@ -28639,7 +28639,7 @@
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>EX-86dd65f493</t>
+          <t>EX-9bb5386d79</t>
         </is>
       </c>
       <c r="B263" s="2" t="inlineStr">
@@ -28689,7 +28689,7 @@
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>EX-86dd65f493</t>
+          <t>EX-9bb5386d79</t>
         </is>
       </c>
       <c r="B264" s="2" t="inlineStr">
@@ -28739,7 +28739,7 @@
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>EX-86dd65f493</t>
+          <t>EX-9bb5386d79</t>
         </is>
       </c>
       <c r="B265" s="2" t="inlineStr">
@@ -28789,7 +28789,7 @@
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>EX-86dd65f493</t>
+          <t>EX-9bb5386d79</t>
         </is>
       </c>
       <c r="B266" s="2" t="inlineStr">
@@ -28839,7 +28839,7 @@
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>EX-86dd65f493</t>
+          <t>EX-9bb5386d79</t>
         </is>
       </c>
       <c r="B267" s="2" t="inlineStr">
@@ -28889,7 +28889,7 @@
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>EX-86dd65f493</t>
+          <t>EX-9bb5386d79</t>
         </is>
       </c>
       <c r="B268" s="2" t="inlineStr">
@@ -28923,7 +28923,7 @@
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>EX-160486754b</t>
+          <t>EX-52ab841ede</t>
         </is>
       </c>
       <c r="B269" s="2" t="inlineStr">
@@ -28973,7 +28973,7 @@
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>EX-160486754b</t>
+          <t>EX-52ab841ede</t>
         </is>
       </c>
       <c r="B270" s="2" t="inlineStr">
@@ -29023,7 +29023,7 @@
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>EX-160486754b</t>
+          <t>EX-52ab841ede</t>
         </is>
       </c>
       <c r="B271" s="2" t="inlineStr">
@@ -29057,7 +29057,7 @@
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>EX-160486754b</t>
+          <t>EX-52ab841ede</t>
         </is>
       </c>
       <c r="B272" s="2" t="inlineStr">
@@ -29107,7 +29107,7 @@
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>EX-160486754b</t>
+          <t>EX-52ab841ede</t>
         </is>
       </c>
       <c r="B273" s="2" t="inlineStr">
@@ -29157,7 +29157,7 @@
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>EX-160486754b</t>
+          <t>EX-52ab841ede</t>
         </is>
       </c>
       <c r="B274" s="2" t="inlineStr">
@@ -29207,7 +29207,7 @@
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>EX-160486754b</t>
+          <t>EX-52ab841ede</t>
         </is>
       </c>
       <c r="B275" s="2" t="inlineStr">
@@ -29257,7 +29257,7 @@
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>EX-160486754b</t>
+          <t>EX-52ab841ede</t>
         </is>
       </c>
       <c r="B276" s="2" t="inlineStr">
@@ -29307,7 +29307,7 @@
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>EX-160486754b</t>
+          <t>EX-52ab841ede</t>
         </is>
       </c>
       <c r="B277" s="2" t="inlineStr">
@@ -29357,7 +29357,7 @@
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>EX-160486754b</t>
+          <t>EX-52ab841ede</t>
         </is>
       </c>
       <c r="B278" s="2" t="inlineStr">
@@ -29407,7 +29407,7 @@
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>EX-160486754b</t>
+          <t>EX-52ab841ede</t>
         </is>
       </c>
       <c r="B279" s="2" t="inlineStr">
@@ -29457,7 +29457,7 @@
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>EX-160486754b</t>
+          <t>EX-52ab841ede</t>
         </is>
       </c>
       <c r="B280" s="2" t="inlineStr">
@@ -29491,7 +29491,7 @@
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>EX-c249fdc70c</t>
+          <t>EX-0dba39ae30</t>
         </is>
       </c>
       <c r="B281" s="2" t="inlineStr">
@@ -29541,7 +29541,7 @@
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>EX-c249fdc70c</t>
+          <t>EX-0dba39ae30</t>
         </is>
       </c>
       <c r="B282" s="2" t="inlineStr">
@@ -29591,7 +29591,7 @@
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>EX-c249fdc70c</t>
+          <t>EX-0dba39ae30</t>
         </is>
       </c>
       <c r="B283" s="2" t="inlineStr">
@@ -29625,7 +29625,7 @@
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>EX-c249fdc70c</t>
+          <t>EX-0dba39ae30</t>
         </is>
       </c>
       <c r="B284" s="2" t="inlineStr">
@@ -29675,7 +29675,7 @@
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>EX-c249fdc70c</t>
+          <t>EX-0dba39ae30</t>
         </is>
       </c>
       <c r="B285" s="2" t="inlineStr">
@@ -29725,7 +29725,7 @@
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>EX-c249fdc70c</t>
+          <t>EX-0dba39ae30</t>
         </is>
       </c>
       <c r="B286" s="2" t="inlineStr">
@@ -29775,7 +29775,7 @@
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>EX-c249fdc70c</t>
+          <t>EX-0dba39ae30</t>
         </is>
       </c>
       <c r="B287" s="2" t="inlineStr">
@@ -29825,7 +29825,7 @@
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>EX-c249fdc70c</t>
+          <t>EX-0dba39ae30</t>
         </is>
       </c>
       <c r="B288" s="2" t="inlineStr">
@@ -29875,7 +29875,7 @@
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>EX-c249fdc70c</t>
+          <t>EX-0dba39ae30</t>
         </is>
       </c>
       <c r="B289" s="2" t="inlineStr">
@@ -29925,7 +29925,7 @@
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>EX-c249fdc70c</t>
+          <t>EX-0dba39ae30</t>
         </is>
       </c>
       <c r="B290" s="2" t="inlineStr">
@@ -29975,7 +29975,7 @@
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>EX-c249fdc70c</t>
+          <t>EX-0dba39ae30</t>
         </is>
       </c>
       <c r="B291" s="2" t="inlineStr">
@@ -30025,7 +30025,7 @@
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>EX-c249fdc70c</t>
+          <t>EX-0dba39ae30</t>
         </is>
       </c>
       <c r="B292" s="2" t="inlineStr">
@@ -30059,7 +30059,7 @@
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>EX-da62ece9dc</t>
+          <t>EX-abb24bea57</t>
         </is>
       </c>
       <c r="B293" s="2" t="inlineStr">
@@ -30109,7 +30109,7 @@
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>EX-da62ece9dc</t>
+          <t>EX-abb24bea57</t>
         </is>
       </c>
       <c r="B294" s="2" t="inlineStr">
@@ -30159,7 +30159,7 @@
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>EX-da62ece9dc</t>
+          <t>EX-abb24bea57</t>
         </is>
       </c>
       <c r="B295" s="2" t="inlineStr">
@@ -30193,7 +30193,7 @@
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>EX-da62ece9dc</t>
+          <t>EX-abb24bea57</t>
         </is>
       </c>
       <c r="B296" s="2" t="inlineStr">
@@ -30243,7 +30243,7 @@
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>EX-da62ece9dc</t>
+          <t>EX-abb24bea57</t>
         </is>
       </c>
       <c r="B297" s="2" t="inlineStr">
@@ -30293,7 +30293,7 @@
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>EX-da62ece9dc</t>
+          <t>EX-abb24bea57</t>
         </is>
       </c>
       <c r="B298" s="2" t="inlineStr">
@@ -30343,7 +30343,7 @@
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>EX-da62ece9dc</t>
+          <t>EX-abb24bea57</t>
         </is>
       </c>
       <c r="B299" s="2" t="inlineStr">
@@ -30393,7 +30393,7 @@
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>EX-da62ece9dc</t>
+          <t>EX-abb24bea57</t>
         </is>
       </c>
       <c r="B300" s="2" t="inlineStr">
@@ -30443,7 +30443,7 @@
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>EX-da62ece9dc</t>
+          <t>EX-abb24bea57</t>
         </is>
       </c>
       <c r="B301" s="2" t="inlineStr">
@@ -30493,7 +30493,7 @@
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>EX-da62ece9dc</t>
+          <t>EX-abb24bea57</t>
         </is>
       </c>
       <c r="B302" s="2" t="inlineStr">
@@ -30543,7 +30543,7 @@
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>EX-da62ece9dc</t>
+          <t>EX-abb24bea57</t>
         </is>
       </c>
       <c r="B303" s="2" t="inlineStr">
@@ -30593,7 +30593,7 @@
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>EX-da62ece9dc</t>
+          <t>EX-abb24bea57</t>
         </is>
       </c>
       <c r="B304" s="2" t="inlineStr">
@@ -30627,7 +30627,7 @@
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>EX-4af3972b89</t>
+          <t>EX-0eaafaa966</t>
         </is>
       </c>
       <c r="B305" s="2" t="inlineStr">
@@ -30677,7 +30677,7 @@
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>EX-4af3972b89</t>
+          <t>EX-0eaafaa966</t>
         </is>
       </c>
       <c r="B306" s="2" t="inlineStr">
@@ -30727,7 +30727,7 @@
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>EX-4af3972b89</t>
+          <t>EX-0eaafaa966</t>
         </is>
       </c>
       <c r="B307" s="2" t="inlineStr">
@@ -30761,7 +30761,7 @@
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>EX-4af3972b89</t>
+          <t>EX-0eaafaa966</t>
         </is>
       </c>
       <c r="B308" s="2" t="inlineStr">
@@ -30807,7 +30807,7 @@
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>EX-4af3972b89</t>
+          <t>EX-0eaafaa966</t>
         </is>
       </c>
       <c r="B309" s="2" t="inlineStr">
@@ -30857,7 +30857,7 @@
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>EX-4af3972b89</t>
+          <t>EX-0eaafaa966</t>
         </is>
       </c>
       <c r="B310" s="2" t="inlineStr">
@@ -30907,7 +30907,7 @@
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>EX-4af3972b89</t>
+          <t>EX-0eaafaa966</t>
         </is>
       </c>
       <c r="B311" s="2" t="inlineStr">
@@ -30957,7 +30957,7 @@
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>EX-4af3972b89</t>
+          <t>EX-0eaafaa966</t>
         </is>
       </c>
       <c r="B312" s="2" t="inlineStr">
@@ -31007,7 +31007,7 @@
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>EX-4af3972b89</t>
+          <t>EX-0eaafaa966</t>
         </is>
       </c>
       <c r="B313" s="2" t="inlineStr">
@@ -31057,7 +31057,7 @@
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>EX-4af3972b89</t>
+          <t>EX-0eaafaa966</t>
         </is>
       </c>
       <c r="B314" s="2" t="inlineStr">
@@ -31107,7 +31107,7 @@
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>EX-4af3972b89</t>
+          <t>EX-0eaafaa966</t>
         </is>
       </c>
       <c r="B315" s="2" t="inlineStr">
@@ -31157,7 +31157,7 @@
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>EX-4af3972b89</t>
+          <t>EX-0eaafaa966</t>
         </is>
       </c>
       <c r="B316" s="2" t="inlineStr">
@@ -31191,7 +31191,7 @@
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>EX-347070bcbc</t>
+          <t>EX-b93f11412e</t>
         </is>
       </c>
       <c r="B317" s="2" t="inlineStr">
@@ -31241,7 +31241,7 @@
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>EX-347070bcbc</t>
+          <t>EX-b93f11412e</t>
         </is>
       </c>
       <c r="B318" s="2" t="inlineStr">
@@ -31291,7 +31291,7 @@
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>EX-347070bcbc</t>
+          <t>EX-b93f11412e</t>
         </is>
       </c>
       <c r="B319" s="2" t="inlineStr">
@@ -31325,7 +31325,7 @@
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>EX-347070bcbc</t>
+          <t>EX-b93f11412e</t>
         </is>
       </c>
       <c r="B320" s="2" t="inlineStr">
@@ -31375,7 +31375,7 @@
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>EX-347070bcbc</t>
+          <t>EX-b93f11412e</t>
         </is>
       </c>
       <c r="B321" s="2" t="inlineStr">
@@ -31421,7 +31421,7 @@
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>EX-347070bcbc</t>
+          <t>EX-b93f11412e</t>
         </is>
       </c>
       <c r="B322" s="2" t="inlineStr">
@@ -31471,7 +31471,7 @@
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>EX-347070bcbc</t>
+          <t>EX-b93f11412e</t>
         </is>
       </c>
       <c r="B323" s="2" t="inlineStr">
@@ -31521,7 +31521,7 @@
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>EX-347070bcbc</t>
+          <t>EX-b93f11412e</t>
         </is>
       </c>
       <c r="B324" s="2" t="inlineStr">
@@ -31571,7 +31571,7 @@
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>EX-347070bcbc</t>
+          <t>EX-b93f11412e</t>
         </is>
       </c>
       <c r="B325" s="2" t="inlineStr">
@@ -31621,7 +31621,7 @@
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>EX-347070bcbc</t>
+          <t>EX-b93f11412e</t>
         </is>
       </c>
       <c r="B326" s="2" t="inlineStr">
@@ -31671,7 +31671,7 @@
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>EX-347070bcbc</t>
+          <t>EX-b93f11412e</t>
         </is>
       </c>
       <c r="B327" s="2" t="inlineStr">
@@ -31721,7 +31721,7 @@
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>EX-347070bcbc</t>
+          <t>EX-b93f11412e</t>
         </is>
       </c>
       <c r="B328" s="2" t="inlineStr">
@@ -31755,7 +31755,7 @@
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>EX-cdf82f12f0</t>
+          <t>EX-f76eb27b5a</t>
         </is>
       </c>
       <c r="B329" s="2" t="inlineStr">
@@ -31805,7 +31805,7 @@
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>EX-cdf82f12f0</t>
+          <t>EX-f76eb27b5a</t>
         </is>
       </c>
       <c r="B330" s="2" t="inlineStr">
@@ -31855,7 +31855,7 @@
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>EX-cdf82f12f0</t>
+          <t>EX-f76eb27b5a</t>
         </is>
       </c>
       <c r="B331" s="2" t="inlineStr">
@@ -31889,7 +31889,7 @@
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>EX-cdf82f12f0</t>
+          <t>EX-f76eb27b5a</t>
         </is>
       </c>
       <c r="B332" s="2" t="inlineStr">
@@ -31939,7 +31939,7 @@
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>EX-cdf82f12f0</t>
+          <t>EX-f76eb27b5a</t>
         </is>
       </c>
       <c r="B333" s="2" t="inlineStr">
@@ -31989,7 +31989,7 @@
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>EX-cdf82f12f0</t>
+          <t>EX-f76eb27b5a</t>
         </is>
       </c>
       <c r="B334" s="2" t="inlineStr">
@@ -32035,7 +32035,7 @@
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>EX-cdf82f12f0</t>
+          <t>EX-f76eb27b5a</t>
         </is>
       </c>
       <c r="B335" s="2" t="inlineStr">
@@ -32085,7 +32085,7 @@
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>EX-cdf82f12f0</t>
+          <t>EX-f76eb27b5a</t>
         </is>
       </c>
       <c r="B336" s="2" t="inlineStr">
@@ -32135,7 +32135,7 @@
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>EX-cdf82f12f0</t>
+          <t>EX-f76eb27b5a</t>
         </is>
       </c>
       <c r="B337" s="2" t="inlineStr">
@@ -32185,7 +32185,7 @@
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>EX-cdf82f12f0</t>
+          <t>EX-f76eb27b5a</t>
         </is>
       </c>
       <c r="B338" s="2" t="inlineStr">
@@ -32235,7 +32235,7 @@
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>EX-cdf82f12f0</t>
+          <t>EX-f76eb27b5a</t>
         </is>
       </c>
       <c r="B339" s="2" t="inlineStr">
@@ -32285,7 +32285,7 @@
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>EX-cdf82f12f0</t>
+          <t>EX-f76eb27b5a</t>
         </is>
       </c>
       <c r="B340" s="2" t="inlineStr">
@@ -32319,7 +32319,7 @@
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>EX-fdc8ce52c7</t>
+          <t>EX-a07af4cf20</t>
         </is>
       </c>
       <c r="B341" s="2" t="inlineStr">
@@ -32369,7 +32369,7 @@
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>EX-fdc8ce52c7</t>
+          <t>EX-a07af4cf20</t>
         </is>
       </c>
       <c r="B342" s="2" t="inlineStr">
@@ -32419,7 +32419,7 @@
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>EX-fdc8ce52c7</t>
+          <t>EX-a07af4cf20</t>
         </is>
       </c>
       <c r="B343" s="2" t="inlineStr">
@@ -32453,7 +32453,7 @@
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>EX-fdc8ce52c7</t>
+          <t>EX-a07af4cf20</t>
         </is>
       </c>
       <c r="B344" s="2" t="inlineStr">
@@ -32503,7 +32503,7 @@
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>EX-fdc8ce52c7</t>
+          <t>EX-a07af4cf20</t>
         </is>
       </c>
       <c r="B345" s="2" t="inlineStr">
@@ -32553,7 +32553,7 @@
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>EX-fdc8ce52c7</t>
+          <t>EX-a07af4cf20</t>
         </is>
       </c>
       <c r="B346" s="2" t="inlineStr">
@@ -32603,7 +32603,7 @@
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>EX-fdc8ce52c7</t>
+          <t>EX-a07af4cf20</t>
         </is>
       </c>
       <c r="B347" s="2" t="inlineStr">
@@ -32645,7 +32645,7 @@
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>EX-fdc8ce52c7</t>
+          <t>EX-a07af4cf20</t>
         </is>
       </c>
       <c r="B348" s="2" t="inlineStr">
@@ -32695,7 +32695,7 @@
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>EX-fdc8ce52c7</t>
+          <t>EX-a07af4cf20</t>
         </is>
       </c>
       <c r="B349" s="2" t="inlineStr">
@@ -32745,7 +32745,7 @@
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>EX-fdc8ce52c7</t>
+          <t>EX-a07af4cf20</t>
         </is>
       </c>
       <c r="B350" s="2" t="inlineStr">
@@ -32795,7 +32795,7 @@
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>EX-fdc8ce52c7</t>
+          <t>EX-a07af4cf20</t>
         </is>
       </c>
       <c r="B351" s="2" t="inlineStr">
@@ -32845,7 +32845,7 @@
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>EX-fdc8ce52c7</t>
+          <t>EX-a07af4cf20</t>
         </is>
       </c>
       <c r="B352" s="2" t="inlineStr">
@@ -32879,7 +32879,7 @@
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>EX-db1b37b406</t>
+          <t>EX-54ee1c0640</t>
         </is>
       </c>
       <c r="B353" s="2" t="inlineStr">
@@ -32929,7 +32929,7 @@
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>EX-db1b37b406</t>
+          <t>EX-54ee1c0640</t>
         </is>
       </c>
       <c r="B354" s="2" t="inlineStr">
@@ -32979,7 +32979,7 @@
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>EX-db1b37b406</t>
+          <t>EX-54ee1c0640</t>
         </is>
       </c>
       <c r="B355" s="2" t="inlineStr">
@@ -33013,7 +33013,7 @@
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>EX-db1b37b406</t>
+          <t>EX-54ee1c0640</t>
         </is>
       </c>
       <c r="B356" s="2" t="inlineStr">
@@ -33063,7 +33063,7 @@
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>EX-db1b37b406</t>
+          <t>EX-54ee1c0640</t>
         </is>
       </c>
       <c r="B357" s="2" t="inlineStr">
@@ -33113,7 +33113,7 @@
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>EX-db1b37b406</t>
+          <t>EX-54ee1c0640</t>
         </is>
       </c>
       <c r="B358" s="2" t="inlineStr">
@@ -33163,7 +33163,7 @@
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>EX-db1b37b406</t>
+          <t>EX-54ee1c0640</t>
         </is>
       </c>
       <c r="B359" s="2" t="inlineStr">
@@ -33213,7 +33213,7 @@
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>EX-db1b37b406</t>
+          <t>EX-54ee1c0640</t>
         </is>
       </c>
       <c r="B360" s="2" t="inlineStr">
@@ -33259,7 +33259,7 @@
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>EX-db1b37b406</t>
+          <t>EX-54ee1c0640</t>
         </is>
       </c>
       <c r="B361" s="2" t="inlineStr">
@@ -33309,7 +33309,7 @@
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>EX-db1b37b406</t>
+          <t>EX-54ee1c0640</t>
         </is>
       </c>
       <c r="B362" s="2" t="inlineStr">
@@ -33359,7 +33359,7 @@
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>EX-db1b37b406</t>
+          <t>EX-54ee1c0640</t>
         </is>
       </c>
       <c r="B363" s="2" t="inlineStr">
@@ -33393,7 +33393,7 @@
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>EX-e98f225bbc</t>
+          <t>EX-34a042894f</t>
         </is>
       </c>
       <c r="B364" s="2" t="inlineStr">
@@ -33443,7 +33443,7 @@
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>EX-e98f225bbc</t>
+          <t>EX-34a042894f</t>
         </is>
       </c>
       <c r="B365" s="2" t="inlineStr">
@@ -33493,7 +33493,7 @@
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>EX-e98f225bbc</t>
+          <t>EX-34a042894f</t>
         </is>
       </c>
       <c r="B366" s="2" t="inlineStr">
@@ -33527,7 +33527,7 @@
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>EX-e98f225bbc</t>
+          <t>EX-34a042894f</t>
         </is>
       </c>
       <c r="B367" s="2" t="inlineStr">
@@ -33577,7 +33577,7 @@
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>EX-e98f225bbc</t>
+          <t>EX-34a042894f</t>
         </is>
       </c>
       <c r="B368" s="2" t="inlineStr">
@@ -33627,7 +33627,7 @@
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>EX-e98f225bbc</t>
+          <t>EX-34a042894f</t>
         </is>
       </c>
       <c r="B369" s="2" t="inlineStr">
@@ -33677,7 +33677,7 @@
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>EX-e98f225bbc</t>
+          <t>EX-34a042894f</t>
         </is>
       </c>
       <c r="B370" s="2" t="inlineStr">
@@ -33727,7 +33727,7 @@
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
         <is>
-          <t>EX-e98f225bbc</t>
+          <t>EX-34a042894f</t>
         </is>
       </c>
       <c r="B371" s="2" t="inlineStr">
@@ -33777,7 +33777,7 @@
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>EX-e98f225bbc</t>
+          <t>EX-34a042894f</t>
         </is>
       </c>
       <c r="B372" s="2" t="inlineStr">
@@ -33823,7 +33823,7 @@
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
         <is>
-          <t>EX-e98f225bbc</t>
+          <t>EX-34a042894f</t>
         </is>
       </c>
       <c r="B373" s="2" t="inlineStr">
@@ -33873,7 +33873,7 @@
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>EX-e98f225bbc</t>
+          <t>EX-34a042894f</t>
         </is>
       </c>
       <c r="B374" s="2" t="inlineStr">
@@ -33923,7 +33923,7 @@
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
         <is>
-          <t>EX-e98f225bbc</t>
+          <t>EX-34a042894f</t>
         </is>
       </c>
       <c r="B375" s="2" t="inlineStr">
@@ -33957,7 +33957,7 @@
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>EX-5e5c61f781</t>
+          <t>EX-0e900c082c</t>
         </is>
       </c>
       <c r="B376" s="2" t="inlineStr">
@@ -34007,7 +34007,7 @@
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
         <is>
-          <t>EX-5e5c61f781</t>
+          <t>EX-0e900c082c</t>
         </is>
       </c>
       <c r="B377" s="2" t="inlineStr">
@@ -34057,7 +34057,7 @@
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>EX-5e5c61f781</t>
+          <t>EX-0e900c082c</t>
         </is>
       </c>
       <c r="B378" s="2" t="inlineStr">
@@ -34091,7 +34091,7 @@
     <row r="379">
       <c r="A379" s="2" t="inlineStr">
         <is>
-          <t>EX-5e5c61f781</t>
+          <t>EX-0e900c082c</t>
         </is>
       </c>
       <c r="B379" s="2" t="inlineStr">
@@ -34141,7 +34141,7 @@
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>EX-5e5c61f781</t>
+          <t>EX-0e900c082c</t>
         </is>
       </c>
       <c r="B380" s="2" t="inlineStr">
@@ -34191,7 +34191,7 @@
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>EX-5e5c61f781</t>
+          <t>EX-0e900c082c</t>
         </is>
       </c>
       <c r="B381" s="2" t="inlineStr">
@@ -34241,7 +34241,7 @@
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>EX-5e5c61f781</t>
+          <t>EX-0e900c082c</t>
         </is>
       </c>
       <c r="B382" s="2" t="inlineStr">
@@ -34291,7 +34291,7 @@
     <row r="383">
       <c r="A383" s="2" t="inlineStr">
         <is>
-          <t>EX-5e5c61f781</t>
+          <t>EX-0e900c082c</t>
         </is>
       </c>
       <c r="B383" s="2" t="inlineStr">
@@ -34341,7 +34341,7 @@
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
-          <t>EX-5e5c61f781</t>
+          <t>EX-0e900c082c</t>
         </is>
       </c>
       <c r="B384" s="2" t="inlineStr">
@@ -34391,7 +34391,7 @@
     <row r="385">
       <c r="A385" s="2" t="inlineStr">
         <is>
-          <t>EX-5e5c61f781</t>
+          <t>EX-0e900c082c</t>
         </is>
       </c>
       <c r="B385" s="2" t="inlineStr">
@@ -34441,7 +34441,7 @@
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
         <is>
-          <t>EX-5e5c61f781</t>
+          <t>EX-0e900c082c</t>
         </is>
       </c>
       <c r="B386" s="2" t="inlineStr">
@@ -34491,7 +34491,7 @@
     <row r="387">
       <c r="A387" s="2" t="inlineStr">
         <is>
-          <t>EX-5e5c61f781</t>
+          <t>EX-0e900c082c</t>
         </is>
       </c>
       <c r="B387" s="2" t="inlineStr">
@@ -34525,7 +34525,7 @@
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
         <is>
-          <t>EX-1295616f39</t>
+          <t>EX-512ea628f4</t>
         </is>
       </c>
       <c r="B388" s="2" t="inlineStr">
@@ -34575,7 +34575,7 @@
     <row r="389">
       <c r="A389" s="2" t="inlineStr">
         <is>
-          <t>EX-1295616f39</t>
+          <t>EX-512ea628f4</t>
         </is>
       </c>
       <c r="B389" s="2" t="inlineStr">
@@ -34625,7 +34625,7 @@
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
         <is>
-          <t>EX-1295616f39</t>
+          <t>EX-512ea628f4</t>
         </is>
       </c>
       <c r="B390" s="2" t="inlineStr">
@@ -34659,7 +34659,7 @@
     <row r="391">
       <c r="A391" s="2" t="inlineStr">
         <is>
-          <t>EX-1295616f39</t>
+          <t>EX-512ea628f4</t>
         </is>
       </c>
       <c r="B391" s="2" t="inlineStr">
@@ -34709,7 +34709,7 @@
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
         <is>
-          <t>EX-1295616f39</t>
+          <t>EX-512ea628f4</t>
         </is>
       </c>
       <c r="B392" s="2" t="inlineStr">
@@ -34759,7 +34759,7 @@
     <row r="393">
       <c r="A393" s="2" t="inlineStr">
         <is>
-          <t>EX-1295616f39</t>
+          <t>EX-512ea628f4</t>
         </is>
       </c>
       <c r="B393" s="2" t="inlineStr">
@@ -34809,7 +34809,7 @@
     <row r="394">
       <c r="A394" s="2" t="inlineStr">
         <is>
-          <t>EX-1295616f39</t>
+          <t>EX-512ea628f4</t>
         </is>
       </c>
       <c r="B394" s="2" t="inlineStr">
@@ -34859,7 +34859,7 @@
     <row r="395">
       <c r="A395" s="2" t="inlineStr">
         <is>
-          <t>EX-1295616f39</t>
+          <t>EX-512ea628f4</t>
         </is>
       </c>
       <c r="B395" s="2" t="inlineStr">
@@ -34909,7 +34909,7 @@
     <row r="396">
       <c r="A396" s="2" t="inlineStr">
         <is>
-          <t>EX-1295616f39</t>
+          <t>EX-512ea628f4</t>
         </is>
       </c>
       <c r="B396" s="2" t="inlineStr">
@@ -34959,7 +34959,7 @@
     <row r="397">
       <c r="A397" s="2" t="inlineStr">
         <is>
-          <t>EX-1295616f39</t>
+          <t>EX-512ea628f4</t>
         </is>
       </c>
       <c r="B397" s="2" t="inlineStr">
@@ -35005,7 +35005,7 @@
     <row r="398">
       <c r="A398" s="2" t="inlineStr">
         <is>
-          <t>EX-1295616f39</t>
+          <t>EX-512ea628f4</t>
         </is>
       </c>
       <c r="B398" s="2" t="inlineStr">
@@ -35055,7 +35055,7 @@
     <row r="399">
       <c r="A399" s="2" t="inlineStr">
         <is>
-          <t>EX-1295616f39</t>
+          <t>EX-512ea628f4</t>
         </is>
       </c>
       <c r="B399" s="2" t="inlineStr">
@@ -35089,7 +35089,7 @@
     <row r="400">
       <c r="A400" s="2" t="inlineStr">
         <is>
-          <t>EX-942b12aff5</t>
+          <t>EX-35f775b75c</t>
         </is>
       </c>
       <c r="B400" s="2" t="inlineStr">
@@ -35139,7 +35139,7 @@
     <row r="401">
       <c r="A401" s="2" t="inlineStr">
         <is>
-          <t>EX-942b12aff5</t>
+          <t>EX-35f775b75c</t>
         </is>
       </c>
       <c r="B401" s="2" t="inlineStr">
@@ -35189,7 +35189,7 @@
     <row r="402">
       <c r="A402" s="2" t="inlineStr">
         <is>
-          <t>EX-942b12aff5</t>
+          <t>EX-35f775b75c</t>
         </is>
       </c>
       <c r="B402" s="2" t="inlineStr">
@@ -35223,7 +35223,7 @@
     <row r="403">
       <c r="A403" s="2" t="inlineStr">
         <is>
-          <t>EX-942b12aff5</t>
+          <t>EX-35f775b75c</t>
         </is>
       </c>
       <c r="B403" s="2" t="inlineStr">
@@ -35273,7 +35273,7 @@
     <row r="404">
       <c r="A404" s="2" t="inlineStr">
         <is>
-          <t>EX-942b12aff5</t>
+          <t>EX-35f775b75c</t>
         </is>
       </c>
       <c r="B404" s="2" t="inlineStr">
@@ -35323,7 +35323,7 @@
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
         <is>
-          <t>EX-942b12aff5</t>
+          <t>EX-35f775b75c</t>
         </is>
       </c>
       <c r="B405" s="2" t="inlineStr">
@@ -35373,7 +35373,7 @@
     <row r="406">
       <c r="A406" s="2" t="inlineStr">
         <is>
-          <t>EX-942b12aff5</t>
+          <t>EX-35f775b75c</t>
         </is>
       </c>
       <c r="B406" s="2" t="inlineStr">
@@ -35423,7 +35423,7 @@
     <row r="407">
       <c r="A407" s="2" t="inlineStr">
         <is>
-          <t>EX-942b12aff5</t>
+          <t>EX-35f775b75c</t>
         </is>
       </c>
       <c r="B407" s="2" t="inlineStr">
@@ -35473,7 +35473,7 @@
     <row r="408">
       <c r="A408" s="2" t="inlineStr">
         <is>
-          <t>EX-942b12aff5</t>
+          <t>EX-35f775b75c</t>
         </is>
       </c>
       <c r="B408" s="2" t="inlineStr">
@@ -35523,7 +35523,7 @@
     <row r="409">
       <c r="A409" s="2" t="inlineStr">
         <is>
-          <t>EX-942b12aff5</t>
+          <t>EX-35f775b75c</t>
         </is>
       </c>
       <c r="B409" s="2" t="inlineStr">
@@ -35573,7 +35573,7 @@
     <row r="410">
       <c r="A410" s="2" t="inlineStr">
         <is>
-          <t>EX-942b12aff5</t>
+          <t>EX-35f775b75c</t>
         </is>
       </c>
       <c r="B410" s="2" t="inlineStr">
@@ -35619,7 +35619,7 @@
     <row r="411">
       <c r="A411" s="2" t="inlineStr">
         <is>
-          <t>EX-942b12aff5</t>
+          <t>EX-35f775b75c</t>
         </is>
       </c>
       <c r="B411" s="2" t="inlineStr">
@@ -35653,7 +35653,7 @@
     <row r="412">
       <c r="A412" s="2" t="inlineStr">
         <is>
-          <t>EX-e07989f4c8</t>
+          <t>EX-0a064a0587</t>
         </is>
       </c>
       <c r="B412" s="2" t="inlineStr">
@@ -35703,7 +35703,7 @@
     <row r="413">
       <c r="A413" s="2" t="inlineStr">
         <is>
-          <t>EX-e07989f4c8</t>
+          <t>EX-0a064a0587</t>
         </is>
       </c>
       <c r="B413" s="2" t="inlineStr">
@@ -35753,7 +35753,7 @@
     <row r="414">
       <c r="A414" s="2" t="inlineStr">
         <is>
-          <t>EX-e07989f4c8</t>
+          <t>EX-0a064a0587</t>
         </is>
       </c>
       <c r="B414" s="2" t="inlineStr">
@@ -35787,7 +35787,7 @@
     <row r="415">
       <c r="A415" s="2" t="inlineStr">
         <is>
-          <t>EX-e07989f4c8</t>
+          <t>EX-0a064a0587</t>
         </is>
       </c>
       <c r="B415" s="2" t="inlineStr">
@@ -35837,7 +35837,7 @@
     <row r="416">
       <c r="A416" s="2" t="inlineStr">
         <is>
-          <t>EX-e07989f4c8</t>
+          <t>EX-0a064a0587</t>
         </is>
       </c>
       <c r="B416" s="2" t="inlineStr">
@@ -35887,7 +35887,7 @@
     <row r="417">
       <c r="A417" s="2" t="inlineStr">
         <is>
-          <t>EX-e07989f4c8</t>
+          <t>EX-0a064a0587</t>
         </is>
       </c>
       <c r="B417" s="2" t="inlineStr">
@@ -35937,7 +35937,7 @@
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
         <is>
-          <t>EX-e07989f4c8</t>
+          <t>EX-0a064a0587</t>
         </is>
       </c>
       <c r="B418" s="2" t="inlineStr">
@@ -35987,7 +35987,7 @@
     <row r="419">
       <c r="A419" s="2" t="inlineStr">
         <is>
-          <t>EX-e07989f4c8</t>
+          <t>EX-0a064a0587</t>
         </is>
       </c>
       <c r="B419" s="2" t="inlineStr">
@@ -36037,7 +36037,7 @@
     <row r="420">
       <c r="A420" s="2" t="inlineStr">
         <is>
-          <t>EX-e07989f4c8</t>
+          <t>EX-0a064a0587</t>
         </is>
       </c>
       <c r="B420" s="2" t="inlineStr">
@@ -36087,7 +36087,7 @@
     <row r="421">
       <c r="A421" s="2" t="inlineStr">
         <is>
-          <t>EX-e07989f4c8</t>
+          <t>EX-0a064a0587</t>
         </is>
       </c>
       <c r="B421" s="2" t="inlineStr">
@@ -36137,7 +36137,7 @@
     <row r="422">
       <c r="A422" s="2" t="inlineStr">
         <is>
-          <t>EX-e07989f4c8</t>
+          <t>EX-0a064a0587</t>
         </is>
       </c>
       <c r="B422" s="2" t="inlineStr">
@@ -36187,7 +36187,7 @@
     <row r="423">
       <c r="A423" s="2" t="inlineStr">
         <is>
-          <t>EX-e07989f4c8</t>
+          <t>EX-0a064a0587</t>
         </is>
       </c>
       <c r="B423" s="2" t="inlineStr">
@@ -36221,7 +36221,7 @@
     <row r="424">
       <c r="A424" s="2" t="inlineStr">
         <is>
-          <t>EX-5dca4371c2</t>
+          <t>EX-c5ee250375</t>
         </is>
       </c>
       <c r="B424" s="2" t="inlineStr">
@@ -36267,7 +36267,7 @@
     <row r="425">
       <c r="A425" s="2" t="inlineStr">
         <is>
-          <t>EX-5dca4371c2</t>
+          <t>EX-c5ee250375</t>
         </is>
       </c>
       <c r="B425" s="2" t="inlineStr">
@@ -36317,7 +36317,7 @@
     <row r="426">
       <c r="A426" s="2" t="inlineStr">
         <is>
-          <t>EX-5dca4371c2</t>
+          <t>EX-c5ee250375</t>
         </is>
       </c>
       <c r="B426" s="2" t="inlineStr">
@@ -36351,7 +36351,7 @@
     <row r="427">
       <c r="A427" s="2" t="inlineStr">
         <is>
-          <t>EX-840491d4e8</t>
+          <t>EX-43db0480fa</t>
         </is>
       </c>
       <c r="B427" s="2" t="inlineStr">
@@ -36401,7 +36401,7 @@
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
         <is>
-          <t>EX-840491d4e8</t>
+          <t>EX-43db0480fa</t>
         </is>
       </c>
       <c r="B428" s="2" t="inlineStr">
@@ -36447,7 +36447,7 @@
     <row r="429">
       <c r="A429" s="2" t="inlineStr">
         <is>
-          <t>EX-840491d4e8</t>
+          <t>EX-43db0480fa</t>
         </is>
       </c>
       <c r="B429" s="2" t="inlineStr">
@@ -36481,7 +36481,7 @@
     <row r="430">
       <c r="A430" s="2" t="inlineStr">
         <is>
-          <t>EX-9ffea583f0</t>
+          <t>EX-f6d89eafba</t>
         </is>
       </c>
       <c r="B430" s="2" t="inlineStr">
@@ -36531,7 +36531,7 @@
     <row r="431">
       <c r="A431" s="2" t="inlineStr">
         <is>
-          <t>EX-9ffea583f0</t>
+          <t>EX-f6d89eafba</t>
         </is>
       </c>
       <c r="B431" s="2" t="inlineStr">
@@ -36581,7 +36581,7 @@
     <row r="432">
       <c r="A432" s="2" t="inlineStr">
         <is>
-          <t>EX-9ffea583f0</t>
+          <t>EX-f6d89eafba</t>
         </is>
       </c>
       <c r="B432" s="2" t="inlineStr">
@@ -36615,7 +36615,7 @@
     <row r="433">
       <c r="A433" s="2" t="inlineStr">
         <is>
-          <t>EX-9ffea583f0</t>
+          <t>EX-f6d89eafba</t>
         </is>
       </c>
       <c r="B433" s="2" t="inlineStr">
@@ -36665,7 +36665,7 @@
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
         <is>
-          <t>EX-9ffea583f0</t>
+          <t>EX-f6d89eafba</t>
         </is>
       </c>
       <c r="B434" s="2" t="inlineStr">
@@ -36715,7 +36715,7 @@
     <row r="435">
       <c r="A435" s="2" t="inlineStr">
         <is>
-          <t>EX-9ffea583f0</t>
+          <t>EX-f6d89eafba</t>
         </is>
       </c>
       <c r="B435" s="2" t="inlineStr">
@@ -36765,7 +36765,7 @@
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
         <is>
-          <t>EX-9ffea583f0</t>
+          <t>EX-f6d89eafba</t>
         </is>
       </c>
       <c r="B436" s="2" t="inlineStr">
@@ -36815,7 +36815,7 @@
     <row r="437">
       <c r="A437" s="2" t="inlineStr">
         <is>
-          <t>EX-9ffea583f0</t>
+          <t>EX-f6d89eafba</t>
         </is>
       </c>
       <c r="B437" s="2" t="inlineStr">
@@ -36865,7 +36865,7 @@
     <row r="438">
       <c r="A438" s="2" t="inlineStr">
         <is>
-          <t>EX-9ffea583f0</t>
+          <t>EX-f6d89eafba</t>
         </is>
       </c>
       <c r="B438" s="2" t="inlineStr">
@@ -36915,7 +36915,7 @@
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
         <is>
-          <t>EX-9ffea583f0</t>
+          <t>EX-f6d89eafba</t>
         </is>
       </c>
       <c r="B439" s="2" t="inlineStr">
@@ -36965,7 +36965,7 @@
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
         <is>
-          <t>EX-9ffea583f0</t>
+          <t>EX-f6d89eafba</t>
         </is>
       </c>
       <c r="B440" s="2" t="inlineStr">
@@ -37015,7 +37015,7 @@
     <row r="441">
       <c r="A441" s="2" t="inlineStr">
         <is>
-          <t>EX-9ffea583f0</t>
+          <t>EX-f6d89eafba</t>
         </is>
       </c>
       <c r="B441" s="2" t="inlineStr">
@@ -37049,7 +37049,7 @@
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
         <is>
-          <t>EX-de17b99f9d</t>
+          <t>EX-30682588ea</t>
         </is>
       </c>
       <c r="B442" s="2" t="inlineStr">
@@ -37099,7 +37099,7 @@
     <row r="443">
       <c r="A443" s="2" t="inlineStr">
         <is>
-          <t>EX-de17b99f9d</t>
+          <t>EX-30682588ea</t>
         </is>
       </c>
       <c r="B443" s="2" t="inlineStr">
@@ -37149,7 +37149,7 @@
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t>EX-de17b99f9d</t>
+          <t>EX-30682588ea</t>
         </is>
       </c>
       <c r="B444" s="2" t="inlineStr">
@@ -37183,7 +37183,7 @@
     <row r="445">
       <c r="A445" s="2" t="inlineStr">
         <is>
-          <t>EX-de17b99f9d</t>
+          <t>EX-30682588ea</t>
         </is>
       </c>
       <c r="B445" s="2" t="inlineStr">
@@ -37233,7 +37233,7 @@
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>EX-de17b99f9d</t>
+          <t>EX-30682588ea</t>
         </is>
       </c>
       <c r="B446" s="2" t="inlineStr">
@@ -37283,7 +37283,7 @@
     <row r="447">
       <c r="A447" s="2" t="inlineStr">
         <is>
-          <t>EX-de17b99f9d</t>
+          <t>EX-30682588ea</t>
         </is>
       </c>
       <c r="B447" s="2" t="inlineStr">
@@ -37333,7 +37333,7 @@
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
         <is>
-          <t>EX-de17b99f9d</t>
+          <t>EX-30682588ea</t>
         </is>
       </c>
       <c r="B448" s="2" t="inlineStr">
@@ -37383,7 +37383,7 @@
     <row r="449">
       <c r="A449" s="2" t="inlineStr">
         <is>
-          <t>EX-de17b99f9d</t>
+          <t>EX-30682588ea</t>
         </is>
       </c>
       <c r="B449" s="2" t="inlineStr">
@@ -37433,7 +37433,7 @@
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>EX-de17b99f9d</t>
+          <t>EX-30682588ea</t>
         </is>
       </c>
       <c r="B450" s="2" t="inlineStr">
@@ -37483,7 +37483,7 @@
     <row r="451">
       <c r="A451" s="2" t="inlineStr">
         <is>
-          <t>EX-de17b99f9d</t>
+          <t>EX-30682588ea</t>
         </is>
       </c>
       <c r="B451" s="2" t="inlineStr">
@@ -37533,7 +37533,7 @@
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
         <is>
-          <t>EX-de17b99f9d</t>
+          <t>EX-30682588ea</t>
         </is>
       </c>
       <c r="B452" s="2" t="inlineStr">
@@ -37583,7 +37583,7 @@
     <row r="453">
       <c r="A453" s="2" t="inlineStr">
         <is>
-          <t>EX-de17b99f9d</t>
+          <t>EX-30682588ea</t>
         </is>
       </c>
       <c r="B453" s="2" t="inlineStr">
@@ -37677,7 +37677,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>EX-e444d15cd5</t>
+          <t>EX-83fb5e05d4</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -37712,7 +37712,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>EX-e444d15cd5</t>
+          <t>EX-83fb5e05d4</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -37749,7 +37749,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>EX-13ff676266</t>
+          <t>EX-4ec3f9bc99</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -37784,7 +37784,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>EX-13ff676266</t>
+          <t>EX-4ec3f9bc99</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -37821,7 +37821,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>EX-36fbba288b</t>
+          <t>EX-5e147c7716</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -37856,7 +37856,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>EX-36fbba288b</t>
+          <t>EX-5e147c7716</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -37893,7 +37893,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>EX-f7fceef0cf</t>
+          <t>EX-afe8f4bfe5</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -37928,7 +37928,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>EX-f7fceef0cf</t>
+          <t>EX-afe8f4bfe5</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -37965,7 +37965,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>EX-a214f02dcd</t>
+          <t>EX-3eb0769072</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -38000,7 +38000,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>EX-a214f02dcd</t>
+          <t>EX-3eb0769072</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -38037,7 +38037,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>EX-f02a205850</t>
+          <t>EX-1e2be181e7</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -38072,7 +38072,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>EX-f02a205850</t>
+          <t>EX-1e2be181e7</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -38109,7 +38109,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>EX-17f2db79d6</t>
+          <t>EX-b24b14d127</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -38144,7 +38144,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>EX-17f2db79d6</t>
+          <t>EX-b24b14d127</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -38171,7 +38171,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>EX-0406c0b88e</t>
+          <t>EX-a99c212c1b</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -38206,7 +38206,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>EX-2f1c4f80c4</t>
+          <t>EX-eefe0eb2e2</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -38241,7 +38241,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>EX-2f1c4f80c4</t>
+          <t>EX-eefe0eb2e2</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -38278,7 +38278,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>EX-49c22f3c37</t>
+          <t>EX-e7c2568040</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -38313,7 +38313,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>EX-49c22f3c37</t>
+          <t>EX-e7c2568040</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -38340,7 +38340,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>EX-cf838aa662</t>
+          <t>EX-40bf3439d5</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -38377,7 +38377,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>EX-10faac68cf</t>
+          <t>EX-704bb186c9</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -38414,7 +38414,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>EX-515f124356</t>
+          <t>EX-a344c1af85</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -38449,7 +38449,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>EX-515f124356</t>
+          <t>EX-a344c1af85</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -38486,7 +38486,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>EX-16ed1bf3d2</t>
+          <t>EX-5ec49d8ac5</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -38521,7 +38521,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>EX-16ed1bf3d2</t>
+          <t>EX-5ec49d8ac5</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -38558,7 +38558,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>EX-80d557c8c4</t>
+          <t>EX-74de97f8b8</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -38585,7 +38585,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>EX-1e9bf99444</t>
+          <t>EX-a46433941c</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -38616,7 +38616,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>EX-1e9bf99444</t>
+          <t>EX-a46433941c</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -38645,7 +38645,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>EX-f7e5521a6e</t>
+          <t>EX-1aff0c29e9</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -38676,7 +38676,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>EX-f7e5521a6e</t>
+          <t>EX-1aff0c29e9</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -38705,7 +38705,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>EX-e3802dba8c</t>
+          <t>EX-4f28a08a75</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -38740,7 +38740,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>EX-8c6e88a595</t>
+          <t>EX-bbd4033aef</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -38775,7 +38775,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>EX-8c6e88a595</t>
+          <t>EX-bbd4033aef</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -38810,7 +38810,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>EX-3fda782b0c</t>
+          <t>EX-3b908df042</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -38845,7 +38845,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>EX-3dc3570d3d</t>
+          <t>EX-4a2a056634</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -38880,7 +38880,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>EX-c43adf7c1c</t>
+          <t>EX-77d29d794c</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -38915,7 +38915,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>EX-30168f639d</t>
+          <t>EX-186eacfa0d</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -38950,7 +38950,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>EX-30168f639d</t>
+          <t>EX-186eacfa0d</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -38985,7 +38985,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>EX-86dd65f493</t>
+          <t>EX-9bb5386d79</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -39020,7 +39020,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>EX-160486754b</t>
+          <t>EX-52ab841ede</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -39055,7 +39055,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>EX-c249fdc70c</t>
+          <t>EX-0dba39ae30</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -39090,7 +39090,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>EX-da62ece9dc</t>
+          <t>EX-abb24bea57</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -39125,7 +39125,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>EX-da62ece9dc</t>
+          <t>EX-abb24bea57</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -39160,7 +39160,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>EX-4af3972b89</t>
+          <t>EX-0eaafaa966</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -39195,7 +39195,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>EX-4af3972b89</t>
+          <t>EX-0eaafaa966</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -39230,7 +39230,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>EX-347070bcbc</t>
+          <t>EX-b93f11412e</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -39265,7 +39265,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>EX-347070bcbc</t>
+          <t>EX-b93f11412e</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -39300,7 +39300,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>EX-cdf82f12f0</t>
+          <t>EX-f76eb27b5a</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -39335,7 +39335,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>EX-cdf82f12f0</t>
+          <t>EX-f76eb27b5a</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -39370,7 +39370,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>EX-fdc8ce52c7</t>
+          <t>EX-a07af4cf20</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -39405,7 +39405,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>EX-fdc8ce52c7</t>
+          <t>EX-a07af4cf20</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -39440,7 +39440,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>EX-db1b37b406</t>
+          <t>EX-54ee1c0640</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -39475,7 +39475,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>EX-db1b37b406</t>
+          <t>EX-54ee1c0640</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -39510,7 +39510,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>EX-e98f225bbc</t>
+          <t>EX-34a042894f</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -39545,7 +39545,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>EX-e98f225bbc</t>
+          <t>EX-34a042894f</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -39580,7 +39580,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>EX-5e5c61f781</t>
+          <t>EX-0e900c082c</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -39615,7 +39615,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>EX-5e5c61f781</t>
+          <t>EX-0e900c082c</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -39650,7 +39650,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>EX-1295616f39</t>
+          <t>EX-512ea628f4</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -39685,7 +39685,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>EX-1295616f39</t>
+          <t>EX-512ea628f4</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -39720,7 +39720,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>EX-942b12aff5</t>
+          <t>EX-35f775b75c</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -39755,7 +39755,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>EX-e07989f4c8</t>
+          <t>EX-0a064a0587</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -39790,7 +39790,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>EX-5dca4371c2</t>
+          <t>EX-c5ee250375</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -39825,7 +39825,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>EX-5dca4371c2</t>
+          <t>EX-c5ee250375</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -39860,7 +39860,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>EX-840491d4e8</t>
+          <t>EX-43db0480fa</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -39895,7 +39895,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>EX-840491d4e8</t>
+          <t>EX-43db0480fa</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -39930,7 +39930,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>EX-9ffea583f0</t>
+          <t>EX-f6d89eafba</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -39967,7 +39967,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>EX-de17b99f9d</t>
+          <t>EX-30682588ea</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -40002,7 +40002,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>EX-de17b99f9d</t>
+          <t>EX-30682588ea</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">

</xml_diff>